<commit_message>
Updated incorrect calculation for DACCS values
</commit_message>
<xml_diff>
--- a/Sensitivity/Harmonization_SAF/Harmonization Sheets/Brazzola_2024_Harmonization.xlsx
+++ b/Sensitivity/Harmonization_SAF/Harmonization Sheets/Brazzola_2024_Harmonization.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr updateLinks="always"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="117" documentId="13_ncr:1_{DB346E89-3769-3B46-A762-B3E18F258ADE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{59CFFD62-9D01-45C3-AC8D-31F3F2E7E2CF}"/>
   <bookViews>
-    <workbookView xWindow="1950" yWindow="1950" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Inputs" sheetId="1" r:id="rId1"/>
@@ -393,7 +393,7 @@
         </row>
         <row r="19">
           <cell r="C19">
-            <v>0.8</v>
+            <v>1.7</v>
           </cell>
         </row>
         <row r="21">
@@ -438,12 +438,12 @@
         </row>
         <row r="33">
           <cell r="C33">
-            <v>1282</v>
+            <v>1371</v>
           </cell>
         </row>
         <row r="34">
           <cell r="C34">
-            <v>480</v>
+            <v>523</v>
           </cell>
         </row>
       </sheetData>
@@ -991,7 +991,7 @@
       </c>
       <c r="C18" s="4">
         <f>[1]Inputs!C19</f>
-        <v>0.8</v>
+        <v>1.7</v>
       </c>
       <c r="D18" t="s">
         <v>21</v>
@@ -1151,7 +1151,7 @@
       </c>
       <c r="C32" s="4">
         <f>[1]Inputs!$C$33</f>
-        <v>1282</v>
+        <v>1371</v>
       </c>
       <c r="D32" t="s">
         <v>29</v>
@@ -1166,7 +1166,7 @@
       </c>
       <c r="C33" s="4">
         <f>[1]Inputs!C34</f>
-        <v>480</v>
+        <v>523</v>
       </c>
       <c r="D33" t="s">
         <v>29</v>
@@ -2439,7 +2439,7 @@
       </c>
       <c r="C2">
         <f>'LCOE Corrected'!C2*Inputs!$C$32/870</f>
-        <v>2148.8094237041387</v>
+        <v>2297.9857409503697</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -2451,7 +2451,7 @@
       </c>
       <c r="C3">
         <f>'LCOE Corrected'!C3*Inputs!$C$32/870</f>
-        <v>1695.0484806647094</v>
+        <v>1812.7234531913543</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -2463,7 +2463,7 @@
       </c>
       <c r="C4">
         <f>'LCOE Corrected'!C4*Inputs!$C$32/870</f>
-        <v>1487.8459888797202</v>
+        <v>1591.1363890437569</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -2475,7 +2475,7 @@
       </c>
       <c r="C5">
         <f>'LCOE Corrected'!C5*Inputs!$C$32/870</f>
-        <v>1359.4065863758051</v>
+        <v>1453.7803665532203</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -2487,7 +2487,7 @@
       </c>
       <c r="C6">
         <f>'LCOE Corrected'!C6*Inputs!$C$32/870</f>
-        <v>1266.5338238023253</v>
+        <v>1354.460118902487</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -2499,7 +2499,7 @@
       </c>
       <c r="C7">
         <f>'LCOE Corrected'!C7*Inputs!$C$32/870</f>
-        <v>1196.2084863799</v>
+        <v>1279.2526012689882</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -2511,7 +2511,7 @@
       </c>
       <c r="C8">
         <f>'LCOE Corrected'!C8*Inputs!$C$32/870</f>
-        <v>1140.2604683560553</v>
+        <v>1219.4205164712573</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -2523,7 +2523,7 @@
       </c>
       <c r="C9">
         <f>'LCOE Corrected'!C9*Inputs!$C$32/870</f>
-        <v>1094.1212117220191</v>
+        <v>1170.0781445170735</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -2535,7 +2535,7 @@
       </c>
       <c r="C10">
         <f>'LCOE Corrected'!C10*Inputs!$C$32/870</f>
-        <v>1055.0139580778734</v>
+        <v>1128.2559567275853</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="C11">
         <f>'LCOE Corrected'!C11*Inputs!$C$32/870</f>
-        <v>1021.1512756969564</v>
+        <v>1092.0424329021273</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -2559,7 +2559,7 @@
       </c>
       <c r="C12">
         <f>'LCOE Corrected'!C12*Inputs!$C$32/870</f>
-        <v>991.64990013755585</v>
+        <v>1060.4929899286967</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -2571,7 +2571,7 @@
       </c>
       <c r="C13">
         <f>'LCOE Corrected'!C13*Inputs!$C$32/870</f>
-        <v>965.34376460327803</v>
+        <v>1032.3606094158301</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -2583,7 +2583,7 @@
       </c>
       <c r="C14">
         <f>'LCOE Corrected'!C14*Inputs!$C$32/870</f>
-        <v>941.64146086170229</v>
+        <v>1007.0128259293242</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="C15">
         <f>'LCOE Corrected'!C15*Inputs!$C$32/870</f>
-        <v>920.10826686983853</v>
+        <v>983.98473781478049</v>
       </c>
     </row>
     <row r="16" spans="1:3">
@@ -2607,7 +2607,7 @@
       </c>
       <c r="C16">
         <f>'LCOE Corrected'!C16*Inputs!$C$32/870</f>
-        <v>900.41639938510934</v>
+        <v>962.92580620669651</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -2619,7 +2619,7 @@
       </c>
       <c r="C17">
         <f>'LCOE Corrected'!C17*Inputs!$C$32/870</f>
-        <v>882.45104513610852</v>
+        <v>943.71324717753885</v>
       </c>
     </row>
     <row r="18" spans="1:3">
@@ -2631,7 +2631,7 @@
       </c>
       <c r="C18">
         <f>'LCOE Corrected'!C18*Inputs!$C$32/870</f>
-        <v>865.86227976822261</v>
+        <v>925.97284365228791</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -2643,7 +2643,7 @@
       </c>
       <c r="C19">
         <f>'LCOE Corrected'!C19*Inputs!$C$32/870</f>
-        <v>850.49043710046283</v>
+        <v>909.53384498029209</v>
       </c>
     </row>
     <row r="20" spans="1:3">
@@ -2655,7 +2655,7 @@
       </c>
       <c r="C20">
         <f>'LCOE Corrected'!C20*Inputs!$C$32/870</f>
-        <v>836.2047386845411</v>
+        <v>894.25639371022294</v>
       </c>
     </row>
     <row r="21" spans="1:3">
@@ -2667,7 +2667,7 @@
       </c>
       <c r="C21">
         <f>'LCOE Corrected'!C21*Inputs!$C$32/870</f>
-        <v>822.89652681514622</v>
+        <v>880.02428881713377</v>
       </c>
     </row>
     <row r="22" spans="1:3">
@@ -2679,7 +2679,7 @@
       </c>
       <c r="C22">
         <f>'LCOE Corrected'!C22*Inputs!$C$32/870</f>
-        <v>810.28691281434942</v>
+        <v>866.53928039662469</v>
       </c>
     </row>
     <row r="23" spans="1:3">
@@ -2691,7 +2691,7 @@
       </c>
       <c r="C23">
         <f>'LCOE Corrected'!C23*Inputs!$C$32/870</f>
-        <v>797.97203921841435</v>
+        <v>853.369474078351</v>
       </c>
     </row>
     <row r="24" spans="1:3">
@@ -2703,7 +2703,7 @@
       </c>
       <c r="C24">
         <f>'LCOE Corrected'!C24*Inputs!$C$32/870</f>
-        <v>785.91463285024474</v>
+        <v>840.47500907775782</v>
       </c>
     </row>
     <row r="25" spans="1:3">
@@ -2715,7 +2715,7 @@
       </c>
       <c r="C25">
         <f>'LCOE Corrected'!C25*Inputs!$C$32/870</f>
-        <v>774.17225619084923</v>
+        <v>827.91744402313134</v>
       </c>
     </row>
     <row r="26" spans="1:3">
@@ -2727,7 +2727,7 @@
       </c>
       <c r="C26">
         <f>'LCOE Corrected'!C26*Inputs!$C$32/870</f>
-        <v>762.74439001085943</v>
+        <v>815.6962236387584</v>
       </c>
     </row>
     <row r="27" spans="1:3">
@@ -2739,7 +2739,7 @@
       </c>
       <c r="C27">
         <f>'LCOE Corrected'!C27*Inputs!$C$32/870</f>
-        <v>751.69744444731839</v>
+        <v>803.88236843781078</v>
       </c>
     </row>
     <row r="28" spans="1:3">
@@ -2751,7 +2751,7 @@
       </c>
       <c r="C28">
         <f>'LCOE Corrected'!C28*Inputs!$C$32/870</f>
-        <v>741.06345832415366</v>
+        <v>792.51014146834211</v>
       </c>
     </row>
     <row r="29" spans="1:3">
@@ -2763,7 +2763,7 @@
       </c>
       <c r="C29">
         <f>'LCOE Corrected'!C29*Inputs!$C$32/870</f>
-        <v>730.86451918192824</v>
+        <v>781.60316364931646</v>
       </c>
     </row>
     <row r="30" spans="1:3">
@@ -2775,7 +2775,7 @@
       </c>
       <c r="C30">
         <f>'LCOE Corrected'!C30*Inputs!$C$32/870</f>
-        <v>721.11453348832322</v>
+        <v>771.176306874018</v>
       </c>
     </row>
     <row r="31" spans="1:3">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="C31">
         <f>'LCOE Corrected'!C31*Inputs!$C$32/870</f>
-        <v>711.82090152349417</v>
+        <v>761.23748517060108</v>
       </c>
     </row>
     <row r="32" spans="1:3">
@@ -2799,7 +2799,7 @@
       </c>
       <c r="C32">
         <f>'LCOE Corrected'!C32*Inputs!$C$32/870</f>
-        <v>747.90647299954708</v>
+        <v>799.82821722494452</v>
       </c>
     </row>
   </sheetData>
@@ -2826,7 +2826,7 @@
       </c>
       <c r="B2">
         <f>'CO2 Cost Corrected'!C2</f>
-        <v>2148.8094237041387</v>
+        <v>2297.9857409503697</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -2835,7 +2835,7 @@
       </c>
       <c r="B3">
         <f>'CO2 Cost Corrected'!C3</f>
-        <v>1695.0484806647094</v>
+        <v>1812.7234531913543</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -2844,7 +2844,7 @@
       </c>
       <c r="B4">
         <f>'CO2 Cost Corrected'!C4</f>
-        <v>1487.8459888797202</v>
+        <v>1591.1363890437569</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -2853,7 +2853,7 @@
       </c>
       <c r="B5">
         <f>'CO2 Cost Corrected'!C5</f>
-        <v>1359.4065863758051</v>
+        <v>1453.7803665532203</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -2862,7 +2862,7 @@
       </c>
       <c r="B6">
         <f>'CO2 Cost Corrected'!C6</f>
-        <v>1266.5338238023253</v>
+        <v>1354.460118902487</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -2871,7 +2871,7 @@
       </c>
       <c r="B7">
         <f>'CO2 Cost Corrected'!C7</f>
-        <v>1196.2084863799</v>
+        <v>1279.2526012689882</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -2880,7 +2880,7 @@
       </c>
       <c r="B8">
         <f>'CO2 Cost Corrected'!C8</f>
-        <v>1140.2604683560553</v>
+        <v>1219.4205164712573</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -2889,7 +2889,7 @@
       </c>
       <c r="B9">
         <f>'CO2 Cost Corrected'!C9</f>
-        <v>1094.1212117220191</v>
+        <v>1170.0781445170735</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -2898,7 +2898,7 @@
       </c>
       <c r="B10">
         <f>'CO2 Cost Corrected'!C10</f>
-        <v>1055.0139580778734</v>
+        <v>1128.2559567275853</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -2907,7 +2907,7 @@
       </c>
       <c r="B11">
         <f>'CO2 Cost Corrected'!C11</f>
-        <v>1021.1512756969564</v>
+        <v>1092.0424329021273</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -2916,7 +2916,7 @@
       </c>
       <c r="B12">
         <f>'CO2 Cost Corrected'!C12</f>
-        <v>991.64990013755585</v>
+        <v>1060.4929899286967</v>
       </c>
     </row>
     <row r="13" spans="1:2">
@@ -2925,7 +2925,7 @@
       </c>
       <c r="B13">
         <f>'CO2 Cost Corrected'!C13</f>
-        <v>965.34376460327803</v>
+        <v>1032.3606094158301</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -2934,7 +2934,7 @@
       </c>
       <c r="B14">
         <f>'CO2 Cost Corrected'!C14</f>
-        <v>941.64146086170229</v>
+        <v>1007.0128259293242</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -2943,7 +2943,7 @@
       </c>
       <c r="B15">
         <f>'CO2 Cost Corrected'!C15</f>
-        <v>920.10826686983853</v>
+        <v>983.98473781478049</v>
       </c>
     </row>
     <row r="16" spans="1:2">
@@ -2952,7 +2952,7 @@
       </c>
       <c r="B16">
         <f>'CO2 Cost Corrected'!C16</f>
-        <v>900.41639938510934</v>
+        <v>962.92580620669651</v>
       </c>
     </row>
     <row r="17" spans="1:2">
@@ -2961,7 +2961,7 @@
       </c>
       <c r="B17">
         <f>'CO2 Cost Corrected'!C17</f>
-        <v>882.45104513610852</v>
+        <v>943.71324717753885</v>
       </c>
     </row>
     <row r="18" spans="1:2">
@@ -2970,7 +2970,7 @@
       </c>
       <c r="B18">
         <f>'CO2 Cost Corrected'!C18</f>
-        <v>865.86227976822261</v>
+        <v>925.97284365228791</v>
       </c>
     </row>
     <row r="19" spans="1:2">
@@ -2979,7 +2979,7 @@
       </c>
       <c r="B19">
         <f>'CO2 Cost Corrected'!C19</f>
-        <v>850.49043710046283</v>
+        <v>909.53384498029209</v>
       </c>
     </row>
     <row r="20" spans="1:2">
@@ -2988,7 +2988,7 @@
       </c>
       <c r="B20">
         <f>'CO2 Cost Corrected'!C20</f>
-        <v>836.2047386845411</v>
+        <v>894.25639371022294</v>
       </c>
     </row>
     <row r="21" spans="1:2">
@@ -2997,7 +2997,7 @@
       </c>
       <c r="B21">
         <f>'CO2 Cost Corrected'!C21</f>
-        <v>822.89652681514622</v>
+        <v>880.02428881713377</v>
       </c>
     </row>
     <row r="22" spans="1:2">
@@ -3006,7 +3006,7 @@
       </c>
       <c r="B22">
         <f>'CO2 Cost Corrected'!C22</f>
-        <v>810.28691281434942</v>
+        <v>866.53928039662469</v>
       </c>
     </row>
     <row r="23" spans="1:2">
@@ -3015,7 +3015,7 @@
       </c>
       <c r="B23">
         <f>'CO2 Cost Corrected'!C23</f>
-        <v>797.97203921841435</v>
+        <v>853.369474078351</v>
       </c>
     </row>
     <row r="24" spans="1:2">
@@ -3024,7 +3024,7 @@
       </c>
       <c r="B24">
         <f>'CO2 Cost Corrected'!C24</f>
-        <v>785.91463285024474</v>
+        <v>840.47500907775782</v>
       </c>
     </row>
     <row r="25" spans="1:2">
@@ -3033,7 +3033,7 @@
       </c>
       <c r="B25">
         <f>'CO2 Cost Corrected'!C25</f>
-        <v>774.17225619084923</v>
+        <v>827.91744402313134</v>
       </c>
     </row>
     <row r="26" spans="1:2">
@@ -3042,7 +3042,7 @@
       </c>
       <c r="B26">
         <f>'CO2 Cost Corrected'!C26</f>
-        <v>762.74439001085943</v>
+        <v>815.6962236387584</v>
       </c>
     </row>
     <row r="27" spans="1:2">
@@ -3051,7 +3051,7 @@
       </c>
       <c r="B27">
         <f>'CO2 Cost Corrected'!C27</f>
-        <v>751.69744444731839</v>
+        <v>803.88236843781078</v>
       </c>
     </row>
     <row r="28" spans="1:2">
@@ -3060,7 +3060,7 @@
       </c>
       <c r="B28">
         <f>'CO2 Cost Corrected'!C28</f>
-        <v>741.06345832415366</v>
+        <v>792.51014146834211</v>
       </c>
     </row>
     <row r="29" spans="1:2">
@@ -3069,7 +3069,7 @@
       </c>
       <c r="B29">
         <f>'CO2 Cost Corrected'!C29</f>
-        <v>730.86451918192824</v>
+        <v>781.60316364931646</v>
       </c>
     </row>
     <row r="30" spans="1:2">
@@ -3078,7 +3078,7 @@
       </c>
       <c r="B30">
         <f>'CO2 Cost Corrected'!C30</f>
-        <v>721.11453348832322</v>
+        <v>771.176306874018</v>
       </c>
     </row>
     <row r="31" spans="1:2">
@@ -3087,7 +3087,7 @@
       </c>
       <c r="B31">
         <f>'CO2 Cost Corrected'!C31</f>
-        <v>711.82090152349417</v>
+        <v>761.23748517060108</v>
       </c>
     </row>
     <row r="32" spans="1:2">
@@ -3096,7 +3096,7 @@
       </c>
       <c r="B32">
         <f>'CO2 Cost Corrected'!C32</f>
-        <v>747.90647299954708</v>
+        <v>799.82821722494452</v>
       </c>
     </row>
   </sheetData>
@@ -3125,7 +3125,7 @@
       </c>
       <c r="B2" s="11">
         <f>'WACC Corrected'!B6</f>
-        <v>1266.5338238023253</v>
+        <v>1354.460118902487</v>
       </c>
       <c r="C2" s="11"/>
       <c r="D2" s="11"/>
@@ -3144,7 +3144,7 @@
       </c>
       <c r="B3" s="9">
         <f>'WACC Corrected'!B32</f>
-        <v>747.90647299954708</v>
+        <v>799.82821722494452</v>
       </c>
       <c r="H3" s="9"/>
       <c r="I3" s="9"/>

</xml_diff>